<commit_message>
Fixed typo in 3-5 and handout
</commit_message>
<xml_diff>
--- a/handouts/chapter_3_5_handout.xlsx
+++ b/handouts/chapter_3_5_handout.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\RData\BYUI-Timeseries-Drafts\handouts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\craigaj\Documents\GitHub\timeseries\handouts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D05534D0-3F38-47D0-8F7F-08C933A74212}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B465143F-F4DC-4A64-804B-87B2061C4DD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CB73943A-C465-40BE-817C-B9991112161C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{CB73943A-C465-40BE-817C-B9991112161C}"/>
   </bookViews>
   <sheets>
     <sheet name="Workbook" sheetId="2" r:id="rId1"/>
@@ -887,10 +887,7 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:sSub>
                       <m:sSubPr>
                         <m:ctrlPr>
@@ -1145,10 +1142,7 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:sSub>
                       <m:sSubPr>
                         <m:ctrlPr>
@@ -1293,10 +1287,7 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:sSub>
                       <m:sSubPr>
                         <m:ctrlPr>
@@ -1496,10 +1487,7 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:sSub>
                       <m:sSubPr>
                         <m:ctrlPr>
@@ -1644,10 +1632,7 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:sSub>
                       <m:sSubPr>
                         <m:ctrlPr>
@@ -2071,20 +2056,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0ABFF2E6-1E13-48EF-9BE3-D6C90C46BEC8}">
   <dimension ref="A1:J92"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="11.88671875" customWidth="1"/>
+    <col min="1" max="2" width="11.90625" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.88671875" customWidth="1"/>
-    <col min="7" max="7" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.6640625" customWidth="1"/>
+    <col min="4" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.90625" customWidth="1"/>
+    <col min="7" max="7" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="48.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="48.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="25" t="s">
         <v>106</v>
       </c>
@@ -2096,7 +2081,7 @@
       <c r="G1" s="26"/>
       <c r="H1" s="27"/>
     </row>
-    <row r="2" spans="1:10" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" ht="30.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -2115,7 +2100,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
         <v>7</v>
       </c>
@@ -2142,7 +2127,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
         <v>9</v>
       </c>
@@ -2169,7 +2154,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
         <v>11</v>
       </c>
@@ -2196,7 +2181,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
         <v>13</v>
       </c>
@@ -2206,7 +2191,9 @@
       <c r="C6" s="11">
         <v>1</v>
       </c>
-      <c r="D6" s="11"/>
+      <c r="D6" s="11">
+        <v>13.7</v>
+      </c>
       <c r="E6" s="11"/>
       <c r="F6" s="11"/>
       <c r="G6" s="11"/>
@@ -2215,7 +2202,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
         <v>15</v>
       </c>
@@ -2241,7 +2228,7 @@
         <v>14.6</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
         <v>17</v>
       </c>
@@ -2267,7 +2254,7 @@
         <v>14.6</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
         <v>19</v>
       </c>
@@ -2293,7 +2280,7 @@
         <v>14.4</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
         <v>21</v>
       </c>
@@ -2319,7 +2306,7 @@
         <v>15.3</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
         <v>23</v>
       </c>
@@ -2337,7 +2324,7 @@
       <c r="G11" s="11"/>
       <c r="H11" s="12"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
         <v>25</v>
       </c>
@@ -2355,7 +2342,7 @@
       <c r="G12" s="11"/>
       <c r="H12" s="12"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
         <v>27</v>
       </c>
@@ -2381,7 +2368,7 @@
         <v>15.5</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="10" t="s">
         <v>29</v>
       </c>
@@ -2407,7 +2394,7 @@
         <v>15.8</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="10" t="s">
         <v>31</v>
       </c>
@@ -2433,7 +2420,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
         <v>33</v>
       </c>
@@ -2459,7 +2446,7 @@
         <v>16.600000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="10" t="s">
         <v>35</v>
       </c>
@@ -2485,7 +2472,7 @@
         <v>16.7</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="10" t="s">
         <v>37</v>
       </c>
@@ -2511,7 +2498,7 @@
         <v>15.1</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="10" t="s">
         <v>39</v>
       </c>
@@ -2537,7 +2524,7 @@
         <v>17.5</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="10" t="s">
         <v>41</v>
       </c>
@@ -2563,7 +2550,7 @@
         <v>17.600000000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="10" t="s">
         <v>43</v>
       </c>
@@ -2589,7 +2576,7 @@
         <v>15.6</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="10" t="s">
         <v>45</v>
       </c>
@@ -2615,7 +2602,7 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="10" t="s">
         <v>47</v>
       </c>
@@ -2641,7 +2628,7 @@
         <v>18.3</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="10" t="s">
         <v>49</v>
       </c>
@@ -2667,7 +2654,7 @@
         <v>16.2</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="10" t="s">
         <v>51</v>
       </c>
@@ -2693,7 +2680,7 @@
         <v>19.600000000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="10" t="s">
         <v>53</v>
       </c>
@@ -2719,7 +2706,7 @@
         <v>19.2</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="10" t="s">
         <v>55</v>
       </c>
@@ -2745,7 +2732,7 @@
         <v>16.600000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="10" t="s">
         <v>57</v>
       </c>
@@ -2771,7 +2758,7 @@
         <v>20.3</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="10" t="s">
         <v>59</v>
       </c>
@@ -2797,7 +2784,7 @@
         <v>19.5</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="10" t="s">
         <v>61</v>
       </c>
@@ -2823,7 +2810,7 @@
         <v>16.2</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="10" t="s">
         <v>63</v>
       </c>
@@ -2849,7 +2836,7 @@
         <v>20.5</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="10" t="s">
         <v>65</v>
       </c>
@@ -2875,7 +2862,7 @@
         <v>19.600000000000001</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" s="10" t="s">
         <v>67</v>
       </c>
@@ -2901,7 +2888,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" s="10" t="s">
         <v>69</v>
       </c>
@@ -2927,7 +2914,7 @@
         <v>20.7</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="s">
         <v>71</v>
       </c>
@@ -2953,7 +2940,7 @@
         <v>19.2</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" s="10" t="s">
         <v>73</v>
       </c>
@@ -2979,7 +2966,7 @@
         <v>15.6</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" s="10" t="s">
         <v>75</v>
       </c>
@@ -3005,7 +2992,7 @@
         <v>19.8</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" s="10" t="s">
         <v>77</v>
       </c>
@@ -3031,7 +3018,7 @@
         <v>18.2</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" s="10" t="s">
         <v>79</v>
       </c>
@@ -3057,7 +3044,7 @@
         <v>14.4</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="10" t="s">
         <v>81</v>
       </c>
@@ -3083,7 +3070,7 @@
         <v>18.7</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" s="10" t="s">
         <v>83</v>
       </c>
@@ -3109,7 +3096,7 @@
         <v>17.3</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" s="10" t="s">
         <v>85</v>
       </c>
@@ -3134,7 +3121,7 @@
       </c>
       <c r="H42" s="12"/>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="10" t="s">
         <v>87</v>
       </c>
@@ -3159,7 +3146,7 @@
       </c>
       <c r="H43" s="12"/>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="10" t="s">
         <v>89</v>
       </c>
@@ -3184,7 +3171,7 @@
       </c>
       <c r="H44" s="12"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="10" t="s">
         <v>91</v>
       </c>
@@ -3209,7 +3196,7 @@
       </c>
       <c r="H45" s="12"/>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="10" t="s">
         <v>93</v>
       </c>
@@ -3235,7 +3222,7 @@
         <v>17.600000000000001</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="10" t="s">
         <v>95</v>
       </c>
@@ -3261,7 +3248,7 @@
         <v>16.100000000000001</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" s="10" t="s">
         <v>97</v>
       </c>
@@ -3287,7 +3274,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" s="10" t="s">
         <v>99</v>
       </c>
@@ -3313,7 +3300,7 @@
         <v>16.899999999999999</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A50" s="13" t="s">
         <v>101</v>
       </c>
@@ -3339,8 +3326,8 @@
         <v>15.5</v>
       </c>
     </row>
-    <row r="91" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="92" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="92" spans="1:2" ht="31.5" x14ac:dyDescent="0.35">
       <c r="A92" s="17" t="s">
         <v>103</v>
       </c>
@@ -3357,23 +3344,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010070F75838E79B0E48B83E8E3F5479A3A2" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2b0c304636f8f537543cd13f583db9d4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xmlns:ns4="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0f089f22c5ce4e61126931f7622145b2" ns3:_="" ns4:_="">
     <xsd:import namespace="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
@@ -3568,32 +3538,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5E1B631-90B0-4D19-A35E-F8DC8BE167A4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C96E0334-A0AA-41B5-AE21-CAD1C9D10746}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBDDC771-C014-4A48-9FCA-802C556EA1D0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3610,4 +3572,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C96E0334-A0AA-41B5-AE21-CAD1C9D10746}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5E1B631-90B0-4D19-A35E-F8DC8BE167A4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>